<commit_message>
Ground Case 03 economics in Glassdoor and public benchmarks
Replace the unsupported salary and unit-cost assumptions with dated Glassdoor, BLS, Unitree, ODRI, and PAL Robotics anchors; add a formula-based financial model, revised downside gates, and refreshed site/QC/Windows release metadata.
</commit_message>
<xml_diff>
--- a/docs/downloads/source/pm-operating-system/excel/ROBOTICS_PM_OPERATING_SYSTEM.xlsx
+++ b/docs/downloads/source/pm-operating-system/excel/ROBOTICS_PM_OPERATING_SYSTEM.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R1237caf8a7f147e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="Rf1e4ed6d87a74279"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="R8c67c2d63c4d4316"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portfolio" sheetId="4" r:id="R81cd3d4e839d4a51"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schedule" sheetId="5" r:id="R1af40a47e5624c6b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RAID" sheetId="6" r:id="Rb294167693ec4c32"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="7" r:id="Rda1001c337874e86"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget_TCO" sheetId="8" r:id="R7f2ee81a7b164878"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benefits" sheetId="9" r:id="R8e872a9581f249ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="10" r:id="Rf6d3067dd3d74e62"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stakeholders" sheetId="11" r:id="R6f91d19b1a624166"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vendors" sheetId="12" r:id="R3323217a864646ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gate_Log" sheetId="13" r:id="Rd2cd6330844a48c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rbfdc0186da2a4b43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R4fd581b8e70b48b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="Rd3224712a2694c55"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portfolio" sheetId="4" r:id="R9a2eb6a6a0fe4a09"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schedule" sheetId="5" r:id="R0172abada51a4b12"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RAID" sheetId="6" r:id="R17e0312b2f374cca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="7" r:id="R3070451fcb134ab0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget_TCO" sheetId="8" r:id="Rcf09a4da05d84079"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benefits" sheetId="9" r:id="R0eb068b0c35248ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="10" r:id="Rf055fbfed8f24bde"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stakeholders" sheetId="11" r:id="R4c582a8149ae4fb3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vendors" sheetId="12" r:id="R922eceff54724bde"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gate_Log" sheetId="13" r:id="R76a7af78fe664adf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -583,7 +583,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R311216b923954747"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5d26b0824b3e4426"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1060,7 +1060,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Evidence-confidence key: PB-H = public benchmark/high; RBE-M = range estimate/medium; SA-L = scenario assumption/low; DC-L = derived calculation/low; UPV = unverified production value.</x:v>
+        <x:v>Evidence-confidence key: PB-H = public benchmark/high; PB-M = public benchmark/medium; RBE-M = research-based estimate/medium; SA-L = scenario assumption/low; DC-L = derived calculation/low; UPV = unverified production value.</x:v>
       </x:c>
       <x:c r="B2" s="7"/>
       <x:c r="C2" s="7"/>
@@ -1155,7 +1155,7 @@
       </x:c>
       <x:c r="H6" s="49" t="n">
         <x:f>SUM(Portfolio!D5:D9)</x:f>
-        <x:v>4792000</x:v>
+        <x:v>4789234</x:v>
       </x:c>
       <x:c r="J6" t="str">
         <x:f>Portfolio!A6</x:f>
@@ -1188,7 +1188,7 @@
       </x:c>
       <x:c r="H7" s="49" t="n">
         <x:f>SUMIF(Portfolio!E5:E9,"&gt;0",Portfolio!E5:E9)</x:f>
-        <x:v>1083505</x:v>
+        <x:v>697375</x:v>
       </x:c>
       <x:c r="J7" t="str">
         <x:f>Portfolio!A7</x:f>
@@ -1196,7 +1196,7 @@
       </x:c>
       <x:c r="K7" t="n">
         <x:f>Portfolio!D7</x:f>
-        <x:v>2400000</x:v>
+        <x:v>2397234</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -1417,9 +1417,9 @@
     <x:mergeCell ref="A10:H10"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc17b6cccc0fc46ba"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c5654ea7ae94fa5"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4ebcf7359ed4767"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R093e34ea1de3481f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1458,7 +1458,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Evidence-confidence key: PB-H = public benchmark/high; RBE-M = range estimate/medium; SA-L = scenario assumption/low; DC-L = derived calculation/low; UPV = unverified production value.</x:v>
+        <x:v>Evidence-confidence key: PB-H = public benchmark/high; PB-M = public benchmark/medium; RBE-M = research-based estimate/medium; SA-L = scenario assumption/low; DC-L = derived calculation/low; UPV = unverified production value.</x:v>
       </x:c>
       <x:c r="B2" s="7"/>
       <x:c r="C2" s="7"/>
@@ -1627,7 +1627,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R255e39a8d461419f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b9ed0dc34514fb7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1666,7 +1666,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Evidence-confidence key: PB-H = public benchmark/high; RBE-M = range estimate/medium; SA-L = scenario assumption/low; DC-L = derived calculation/low; UPV = unverified production value.</x:v>
+        <x:v>Evidence-confidence key: PB-H = public benchmark/high; PB-M = public benchmark/medium; RBE-M = research-based estimate/medium; SA-L = scenario assumption/low; DC-L = derived calculation/low; UPV = unverified production value.</x:v>
       </x:c>
       <x:c r="B2" s="7"/>
       <x:c r="C2" s="7"/>
@@ -1826,7 +1826,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R087cfc94b9d34887"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45e452bed4ba47f1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1863,7 +1863,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Evidence-confidence key: PB-H = public benchmark/high; RBE-M = range estimate/medium; SA-L = scenario assumption/low; DC-L = derived calculation/low; UPV = unverified production value.</x:v>
+        <x:v>Evidence-confidence key: PB-H = public benchmark/high; PB-M = public benchmark/medium; RBE-M = research-based estimate/medium; SA-L = scenario assumption/low; DC-L = derived calculation/low; UPV = unverified production value.</x:v>
       </x:c>
       <x:c r="B2" s="7"/>
       <x:c r="C2" s="7"/>
@@ -2015,7 +2015,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96bd336cce2546d7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf3c97b676f2b4e7e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2054,7 +2054,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Evidence-confidence key: PB-H = public benchmark/high; RBE-M = range estimate/medium; SA-L = scenario assumption/low; DC-L = derived calculation/low; UPV = unverified production value.</x:v>
+        <x:v>Evidence-confidence key: PB-H = public benchmark/high; PB-M = public benchmark/medium; RBE-M = research-based estimate/medium; SA-L = scenario assumption/low; DC-L = derived calculation/low; UPV = unverified production value.</x:v>
       </x:c>
       <x:c r="B2" s="7"/>
       <x:c r="C2" s="7"/>
@@ -2293,7 +2293,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8842df990bef4a86"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1aed1a4968bc4813"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2318,7 +2318,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Evidence-confidence key: PB-H = public benchmark/high; RBE-M = range estimate/medium; SA-L = scenario assumption/low; DC-L = derived calculation/low; UPV = unverified production value.</x:v>
+        <x:v>Evidence-confidence key: PB-H = public benchmark/high; PB-M = public benchmark/medium; RBE-M = research-based estimate/medium; SA-L = scenario assumption/low; DC-L = derived calculation/low; UPV = unverified production value.</x:v>
       </x:c>
       <x:c r="B2" s="7"/>
       <x:c r="C2" s="7"/>
@@ -2415,7 +2415,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra7cc38a84e8f434c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re5bb2aa730a74f7c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2452,7 +2452,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Evidence-confidence key: PB-H = public benchmark/high; RBE-M = range estimate/medium; SA-L = scenario assumption/low; DC-L = derived calculation/low; UPV = unverified production value.</x:v>
+        <x:v>Evidence-confidence key: PB-H = public benchmark/high; PB-M = public benchmark/medium; RBE-M = research-based estimate/medium; SA-L = scenario assumption/low; DC-L = derived calculation/low; UPV = unverified production value.</x:v>
       </x:c>
       <x:c r="B2" s="7"/>
       <x:c r="C2" s="7"/>
@@ -2604,7 +2604,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8b81cd16b3b4a25"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3164b99451f64924"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2641,7 +2641,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Evidence-confidence key: PB-H = public benchmark/high; RBE-M = range estimate/medium; SA-L = scenario assumption/low; DC-L = derived calculation/low; UPV = unverified production value.</x:v>
+        <x:v>Evidence-confidence key: PB-H = public benchmark/high; PB-M = public benchmark/medium; RBE-M = research-based estimate/medium; SA-L = scenario assumption/low; DC-L = derived calculation/low; UPV = unverified production value.</x:v>
       </x:c>
       <x:c r="B2" s="7"/>
       <x:c r="C2" s="7"/>
@@ -2760,25 +2760,25 @@
         <x:v>Productization</x:v>
       </x:c>
       <x:c r="D7" s="34" t="n">
-        <x:v>2400000</x:v>
+        <x:v>2397234</x:v>
       </x:c>
       <x:c r="E7" s="34" t="n">
-        <x:v>412800</x:v>
+        <x:v>26670</x:v>
       </x:c>
       <x:c r="F7" s="29" t="str">
-        <x:v>41 robots recover productization authorization</x:v>
+        <x:v>48 robots recover modeled productization authorization</x:v>
       </x:c>
       <x:c r="G7" s="29" t="str">
         <x:v>Conditional</x:v>
       </x:c>
       <x:c r="H7" s="29" t="str">
-        <x:v>SA-L/DC-L</x:v>
+        <x:v>PB-H/PB-M/SA-L/DC-L</x:v>
       </x:c>
       <x:c r="I7" s="29" t="str">
         <x:v>Low</x:v>
       </x:c>
       <x:c r="J7" s="30" t="str">
-        <x:v>Case 03 unit economics and open-source gates</x:v>
+        <x:v>Glassdoor, BLS, Unitree, and disclosed assumptions</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -2861,7 +2861,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73c846e08def4c08"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ebb52bfe54b44ce"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2904,7 +2904,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Evidence-confidence key: PB-H = public benchmark/high; RBE-M = range estimate/medium; SA-L = scenario assumption/low; DC-L = derived calculation/low; UPV = unverified production value.</x:v>
+        <x:v>Evidence-confidence key: PB-H = public benchmark/high; PB-M = public benchmark/medium; RBE-M = research-based estimate/medium; SA-L = scenario assumption/low; DC-L = derived calculation/low; UPV = unverified production value.</x:v>
       </x:c>
       <x:c r="B2" s="7"/>
       <x:c r="C2" s="7"/>
@@ -3179,7 +3179,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b93fc9da875402c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R903c6fc7b7be4e05"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3224,7 +3224,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Evidence-confidence key: PB-H = public benchmark/high; RBE-M = range estimate/medium; SA-L = scenario assumption/low; DC-L = derived calculation/low; UPV = unverified production value.</x:v>
+        <x:v>Evidence-confidence key: PB-H = public benchmark/high; PB-M = public benchmark/medium; RBE-M = research-based estimate/medium; SA-L = scenario assumption/low; DC-L = derived calculation/low; UPV = unverified production value.</x:v>
       </x:c>
       <x:c r="B2" s="7"/>
       <x:c r="C2" s="7"/>
@@ -3437,7 +3437,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83f52495eef9472d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rca59b6b84ac84639"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3478,7 +3478,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Evidence-confidence key: PB-H = public benchmark/high; RBE-M = range estimate/medium; SA-L = scenario assumption/low; DC-L = derived calculation/low; UPV = unverified production value.</x:v>
+        <x:v>Evidence-confidence key: PB-H = public benchmark/high; PB-M = public benchmark/medium; RBE-M = research-based estimate/medium; SA-L = scenario assumption/low; DC-L = derived calculation/low; UPV = unverified production value.</x:v>
       </x:c>
       <x:c r="B2" s="7"/>
       <x:c r="C2" s="7"/>
@@ -3660,7 +3660,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2b1d883cb8cf44c8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ba3cf411353488e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3701,7 +3701,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Evidence-confidence key: PB-H = public benchmark/high; RBE-M = range estimate/medium; SA-L = scenario assumption/low; DC-L = derived calculation/low; UPV = unverified production value.</x:v>
+        <x:v>Evidence-confidence key: PB-H = public benchmark/high; PB-M = public benchmark/medium; RBE-M = research-based estimate/medium; SA-L = scenario assumption/low; DC-L = derived calculation/low; UPV = unverified production value.</x:v>
       </x:c>
       <x:c r="B2" s="7"/>
       <x:c r="C2" s="7"/>
@@ -3921,7 +3921,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb64e7f0e279f4551"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c8efff5d380409c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3964,7 +3964,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Evidence-confidence key: PB-H = public benchmark/high; RBE-M = range estimate/medium; SA-L = scenario assumption/low; DC-L = derived calculation/low; UPV = unverified production value.</x:v>
+        <x:v>Evidence-confidence key: PB-H = public benchmark/high; PB-M = public benchmark/medium; RBE-M = research-based estimate/medium; SA-L = scenario assumption/low; DC-L = derived calculation/low; UPV = unverified production value.</x:v>
       </x:c>
       <x:c r="B2" s="7"/>
       <x:c r="C2" s="7"/>
@@ -4155,7 +4155,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R65ea1edf057d4e66"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2db2b67dcdc840d9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>